<commit_message>
week 02 - after lecture
</commit_message>
<xml_diff>
--- a/Week 02/Python basics/Exported data/Runner data.xlsx
+++ b/Week 02/Python basics/Exported data/Runner data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -448,7 +448,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>first name</t>
+          <t>First name</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -465,7 +465,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>last name</t>
+          <t>Last name</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -482,7 +482,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>full name</t>
+          <t>Full name</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -525,6 +525,23 @@
       <c r="C6" t="inlineStr">
         <is>
           <t>list</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>http://usainbolt.com</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>str</t>
         </is>
       </c>
     </row>

</xml_diff>